<commit_message>
Fix the swapped headers in WT_cAMP_vs_TRUPATH_All_Drugs.xlsx at source
The two Emax columns were mislabelled, and five scripts each compensated for it
with their own comment. Verified against param_table.csv which column is which:
the column labelled 'cAMP Response' matches the published TRUPATH Gi1 Emax to
0.05, and 'TRUPATH (Gi1)' is the raw cAMP span, reproducing the published cAMP
Emax to 0.05 once divided by DAMGO's.

Renamed to TRUPATH_Gi1_Emax_pct_DAMGO and cAMP_response_raw, and updated all
twelve consumers across both repositories. Figure 5f still reproduces
Spearman rho = -0.96 with naloxone at 14.9% and DAMGO at 100%.

Removes the caveat from data/README.md and regenerates MANIFEST.sha256.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/pharmacology/WT_cAMP_vs_TRUPATH_All_Drugs.xlsx
+++ b/data/pharmacology/WT_cAMP_vs_TRUPATH_All_Drugs.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,36 +25,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002F4F4F"/>
-        <bgColor rgb="002F4F4F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F9F9F9"/>
-        <bgColor rgb="00F9F9F9"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -62,41 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D3D3D3"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D3D3D3"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D3D3D3"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D3D3D3"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -464,193 +415,188 @@
   </sheetPr>
   <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Ligand</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>cAMP Response</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>TRUPATH (Gi1)</t>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TRUPATH_Gi1_Emax_pct_DAMGO</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>cAMP_response_raw</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>DAMGO</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" t="n">
         <v>100</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" t="n">
         <v>-0.6159</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>PZM21</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" t="n">
         <v>78.72</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" t="n">
         <v>-0.5987</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Methadone</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" t="n">
         <v>83.33</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" t="n">
         <v>-0.5685</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Naloxone</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" t="n">
         <v>14.88</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" t="n">
         <v>-0.1303</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Carfentanil</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" t="n">
         <v>97.15000000000001</v>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C6" t="n">
         <v>-0.6348</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Morphine</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" t="n">
         <v>98.77</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" t="n">
         <v>-0.5492</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Nalbuphine</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" t="n">
         <v>46.96</v>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" t="n">
         <v>-0.4038</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Butorphanol</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" t="n">
         <v>64.81</v>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C9" t="n">
         <v>-0.4571</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Buprenorphine</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" t="n">
         <v>60.18</v>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C10" t="n">
         <v>-0.2713</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>C6Guano</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B11" t="n">
         <v>88.31999999999999</v>
       </c>
-      <c r="C11" s="3" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>TRV130</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" t="n">
         <v>77.20999999999999</v>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="C12" t="n">
         <v>-0.6347</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>MP</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B13" t="n">
         <v>65.92</v>
       </c>
-      <c r="C13" s="3" t="n">
+      <c r="C13" t="n">
         <v>-0.578</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Fentanyl</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B14" t="n">
         <v>96.39</v>
       </c>
-      <c r="C14" s="2" t="n">
+      <c r="C14" t="n">
         <v>-0.6113</v>
       </c>
     </row>

</xml_diff>